<commit_message>
Tracker: add Collect tab (recurring docs x years per hotel: where kept / missing)
</commit_message>
<xml_diff>
--- a/output/License_Contract_Tracker_4properties.xlsx
+++ b/output/License_Contract_Tracker_4properties.xlsx
@@ -13,8 +13,9 @@
     <sheet name="AES" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="LYF" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="SP" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Feed" sheetId="7" state="hidden" r:id="rId7"/>
-    <sheet name="Lists" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Collect" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Feed" sheetId="8" state="hidden" r:id="rId8"/>
+    <sheet name="Lists" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SR9'!$A$4:$S$124</definedName>
@@ -31,7 +32,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="DD-MMM-YYYY"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,11 +60,15 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="00595959"/>
+      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F3864"/>
-      <sz val="12"/>
     </font>
     <font>
       <i val="1"/>
@@ -202,7 +207,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -212,9 +217,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -226,29 +231,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -268,22 +273,22 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -301,12 +306,18 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="8">
     <dxf>
       <font>
         <b val="1"/>
@@ -378,6 +389,13 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00EDEDED"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF2CC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -743,7 +761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:C24"/>
+  <dimension ref="B1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -941,22 +959,46 @@
     <row r="23" ht="30" customHeight="1">
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Hidden tab 'Feed'</t>
+          <t>Collect tab</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>A hidden helper that joins the 4 hotel tabs for the Dashboard's expiring-next list. Leave it be.</t>
+          <t>The completeness check: one line per recurring document, one column per year, per hotel. Type WHERE that year's copy is kept (ATB / Mitsui / Data room) — it turns green. Type 'Missing' if it cannot be found (red), 'N/A' if that year does not apply (grey). Blank = not checked yet (amber).</t>
         </is>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="B24" s="2" t="inlineStr">
         <is>
+          <t>แท็บ Collect</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>เช็คว่าเอกสารย้อนหลังครบไหม พิมพ์ที่เก็บลงช่องปี (เขียว=มี, Missing=หาย, N/A=ไม่เกี่ยว, ว่าง=ยังไม่เช็ค)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Hidden tab 'Feed'</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>A hidden helper that joins the 4 hotel tabs for the Dashboard's expiring-next list. Leave it be.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="B26" s="2" t="inlineStr">
+        <is>
           <t>Rebuild</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>scripts/build_license_tracker.py rebuilds this file's structure from empty rows — never overwrite a filled-in copy.</t>
         </is>
@@ -29790,6 +29832,2234 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:M74"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Document Collection Check — มีครบไหม เก็บที่ไหน</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>One line per recurring document, one column per year. In each box type WHERE it is kept (ATB / Mitsui / Data room…) — green = have. Type Missing = red, N/A = grey (e.g. before opening). Blank = not checked yet. พิมพ์ที่เก็บเอกสารลงช่องปี ถ้าหาย พิมพ์ Missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="6" customHeight="1"/>
+    <row r="4">
+      <c r="A4" s="44" t="inlineStr">
+        <is>
+          <t>1. SR9 — Somerset Rama 9 Bangkok</t>
+        </is>
+      </c>
+      <c r="B4" s="45" t="n"/>
+      <c r="C4" s="45" t="n"/>
+      <c r="D4" s="45" t="n"/>
+      <c r="E4" s="45" t="n"/>
+      <c r="F4" s="45" t="n"/>
+      <c r="G4" s="45" t="n"/>
+      <c r="H4" s="45" t="n"/>
+      <c r="I4" s="45" t="n"/>
+      <c r="J4" s="45" t="n"/>
+      <c r="K4" s="45" t="n"/>
+      <c r="L4" s="45" t="n"/>
+      <c r="M4" s="45" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="46" t="inlineStr">
+        <is>
+          <t>Document</t>
+        </is>
+      </c>
+      <c r="B5" s="46" t="inlineStr">
+        <is>
+          <t>เอกสาร</t>
+        </is>
+      </c>
+      <c r="C5" s="46" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D5" s="46" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="E5" s="46" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="F5" s="46" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="G5" s="46" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="H5" s="46" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I5" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="J5" s="46" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="K5" s="46" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="L5" s="46" t="inlineStr">
+        <is>
+          <t>Have</t>
+        </is>
+      </c>
+      <c r="M5" s="46" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>EIA monitoring report — 1H</t>
+        </is>
+      </c>
+      <c r="B6" s="47" t="inlineStr">
+        <is>
+          <t>รายงานติดตาม EIA — ครึ่งปีแรก</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="n"/>
+      <c r="D6" s="12" t="n"/>
+      <c r="E6" s="12" t="n"/>
+      <c r="F6" s="12" t="n"/>
+      <c r="G6" s="12" t="n"/>
+      <c r="H6" s="12" t="n"/>
+      <c r="I6" s="12" t="n"/>
+      <c r="J6" s="12" t="n"/>
+      <c r="K6" s="12" t="n"/>
+      <c r="L6" s="12">
+        <f>COUNTIF(C6:K6,"?*")-COUNTIF(C6:K6,"Missing")-COUNTIF(C6:K6,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M6" s="12">
+        <f>COUNTIF(C6:K6,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>EIA monitoring report — 2H</t>
+        </is>
+      </c>
+      <c r="B7" s="47" t="inlineStr">
+        <is>
+          <t>รายงานติดตาม EIA — ครึ่งปีหลัง</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="n"/>
+      <c r="D7" s="12" t="n"/>
+      <c r="E7" s="12" t="n"/>
+      <c r="F7" s="12" t="n"/>
+      <c r="G7" s="12" t="n"/>
+      <c r="H7" s="12" t="n"/>
+      <c r="I7" s="12" t="n"/>
+      <c r="J7" s="12" t="n"/>
+      <c r="K7" s="12" t="n"/>
+      <c r="L7" s="12">
+        <f>COUNTIF(C7:K7,"?*")-COUNTIF(C7:K7,"Missing")-COUNTIF(C7:K7,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M7" s="12">
+        <f>COUNTIF(C7:K7,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Annual building inspection (Ror.1)</t>
+        </is>
+      </c>
+      <c r="B8" s="47" t="inlineStr">
+        <is>
+          <t>รายงานตรวจสอบอาคาร (ร.1)</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="n"/>
+      <c r="D8" s="12" t="n"/>
+      <c r="E8" s="12" t="n"/>
+      <c r="F8" s="12" t="n"/>
+      <c r="G8" s="12" t="n"/>
+      <c r="H8" s="12" t="n"/>
+      <c r="I8" s="12" t="n"/>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="12" t="n"/>
+      <c r="L8" s="12">
+        <f>COUNTIF(C8:K8,"?*")-COUNTIF(C8:K8,"Missing")-COUNTIF(C8:K8,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M8" s="12">
+        <f>COUNTIF(C8:K8,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Workplace environment assessment</t>
+        </is>
+      </c>
+      <c r="B9" s="47" t="inlineStr">
+        <is>
+          <t>ผลตรวจวัดสภาพแวดล้อมในการทำงาน</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="n"/>
+      <c r="D9" s="12" t="n"/>
+      <c r="E9" s="12" t="n"/>
+      <c r="F9" s="12" t="n"/>
+      <c r="G9" s="12" t="n"/>
+      <c r="H9" s="12" t="n"/>
+      <c r="I9" s="12" t="n"/>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="12" t="n"/>
+      <c r="L9" s="12">
+        <f>COUNTIF(C9:K9,"?*")-COUNTIF(C9:K9,"Missing")-COUNTIF(C9:K9,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M9" s="12">
+        <f>COUNTIF(C9:K9,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Air / water / wastewater test reports</t>
+        </is>
+      </c>
+      <c r="B10" s="47" t="inlineStr">
+        <is>
+          <t>ผลตรวจอากาศ น้ำ น้ำทิ้ง</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="n"/>
+      <c r="D10" s="12" t="n"/>
+      <c r="E10" s="12" t="n"/>
+      <c r="F10" s="12" t="n"/>
+      <c r="G10" s="12" t="n"/>
+      <c r="H10" s="12" t="n"/>
+      <c r="I10" s="12" t="n"/>
+      <c r="J10" s="12" t="n"/>
+      <c r="K10" s="12" t="n"/>
+      <c r="L10" s="12">
+        <f>COUNTIF(C10:K10,"?*")-COUNTIF(C10:K10,"Missing")-COUNTIF(C10:K10,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M10" s="12">
+        <f>COUNTIF(C10:K10,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Land &amp; building tax receipt</t>
+        </is>
+      </c>
+      <c r="B11" s="47" t="inlineStr">
+        <is>
+          <t>ใบเสร็จภาษีที่ดินและสิ่งปลูกสร้าง</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="n"/>
+      <c r="D11" s="12" t="n"/>
+      <c r="E11" s="12" t="n"/>
+      <c r="F11" s="12" t="n"/>
+      <c r="G11" s="12" t="n"/>
+      <c r="H11" s="12" t="n"/>
+      <c r="I11" s="12" t="n"/>
+      <c r="J11" s="12" t="n"/>
+      <c r="K11" s="12" t="n"/>
+      <c r="L11" s="12">
+        <f>COUNTIF(C11:K11,"?*")-COUNTIF(C11:K11,"Missing")-COUNTIF(C11:K11,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M11" s="12">
+        <f>COUNTIF(C11:K11,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Signage tax receipt</t>
+        </is>
+      </c>
+      <c r="B12" s="47" t="inlineStr">
+        <is>
+          <t>ใบเสร็จภาษีป้าย</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="12" t="n"/>
+      <c r="F12" s="12" t="n"/>
+      <c r="G12" s="12" t="n"/>
+      <c r="H12" s="12" t="n"/>
+      <c r="I12" s="12" t="n"/>
+      <c r="J12" s="12" t="n"/>
+      <c r="K12" s="12" t="n"/>
+      <c r="L12" s="12">
+        <f>COUNTIF(C12:K12,"?*")-COUNTIF(C12:K12,"Missing")-COUNTIF(C12:K12,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M12" s="12">
+        <f>COUNTIF(C12:K12,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Audited FS (EN)</t>
+        </is>
+      </c>
+      <c r="B13" s="47" t="inlineStr">
+        <is>
+          <t>งบการเงินตรวจสอบแล้ว (อังกฤษ)</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="n"/>
+      <c r="D13" s="12" t="n"/>
+      <c r="E13" s="12" t="n"/>
+      <c r="F13" s="12" t="n"/>
+      <c r="G13" s="12" t="n"/>
+      <c r="H13" s="12" t="n"/>
+      <c r="I13" s="12" t="n"/>
+      <c r="J13" s="12" t="n"/>
+      <c r="K13" s="12" t="n"/>
+      <c r="L13" s="12">
+        <f>COUNTIF(C13:K13,"?*")-COUNTIF(C13:K13,"Missing")-COUNTIF(C13:K13,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M13" s="12">
+        <f>COUNTIF(C13:K13,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Audited FS (TH)</t>
+        </is>
+      </c>
+      <c r="B14" s="47" t="inlineStr">
+        <is>
+          <t>งบการเงินตรวจสอบแล้ว (ไทย)</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="n"/>
+      <c r="D14" s="12" t="n"/>
+      <c r="E14" s="12" t="n"/>
+      <c r="F14" s="12" t="n"/>
+      <c r="G14" s="12" t="n"/>
+      <c r="H14" s="12" t="n"/>
+      <c r="I14" s="12" t="n"/>
+      <c r="J14" s="12" t="n"/>
+      <c r="K14" s="12" t="n"/>
+      <c r="L14" s="12">
+        <f>COUNTIF(C14:K14,"?*")-COUNTIF(C14:K14,"Missing")-COUNTIF(C14:K14,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M14" s="12">
+        <f>COUNTIF(C14:K14,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>PND.50 filing</t>
+        </is>
+      </c>
+      <c r="B15" s="47" t="inlineStr">
+        <is>
+          <t>แบบ ภ.ง.ด.50</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="n"/>
+      <c r="D15" s="12" t="n"/>
+      <c r="E15" s="12" t="n"/>
+      <c r="F15" s="12" t="n"/>
+      <c r="G15" s="12" t="n"/>
+      <c r="H15" s="12" t="n"/>
+      <c r="I15" s="12" t="n"/>
+      <c r="J15" s="12" t="n"/>
+      <c r="K15" s="12" t="n"/>
+      <c r="L15" s="12">
+        <f>COUNTIF(C15:K15,"?*")-COUNTIF(C15:K15,"Missing")-COUNTIF(C15:K15,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M15" s="12">
+        <f>COUNTIF(C15:K15,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>PND.51 filing</t>
+        </is>
+      </c>
+      <c r="B16" s="47" t="inlineStr">
+        <is>
+          <t>แบบ ภ.ง.ด.51</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="n"/>
+      <c r="D16" s="12" t="n"/>
+      <c r="E16" s="12" t="n"/>
+      <c r="F16" s="12" t="n"/>
+      <c r="G16" s="12" t="n"/>
+      <c r="H16" s="12" t="n"/>
+      <c r="I16" s="12" t="n"/>
+      <c r="J16" s="12" t="n"/>
+      <c r="K16" s="12" t="n"/>
+      <c r="L16" s="12">
+        <f>COUNTIF(C16:K16,"?*")-COUNTIF(C16:K16,"Missing")-COUNTIF(C16:K16,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M16" s="12">
+        <f>COUNTIF(C16:K16,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>Insurance policy set (IAR / BI / PV)</t>
+        </is>
+      </c>
+      <c r="B17" s="47" t="inlineStr">
+        <is>
+          <t>กรมธรรม์ประกันทรัพย์สินชุดปี</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="n"/>
+      <c r="D17" s="12" t="n"/>
+      <c r="E17" s="12" t="n"/>
+      <c r="F17" s="12" t="n"/>
+      <c r="G17" s="12" t="n"/>
+      <c r="H17" s="12" t="n"/>
+      <c r="I17" s="12" t="n"/>
+      <c r="J17" s="12" t="n"/>
+      <c r="K17" s="12" t="n"/>
+      <c r="L17" s="12">
+        <f>COUNTIF(C17:K17,"?*")-COUNTIF(C17:K17,"Missing")-COUNTIF(C17:K17,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M17" s="12">
+        <f>COUNTIF(C17:K17,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>Public liability policy</t>
+        </is>
+      </c>
+      <c r="B18" s="47" t="inlineStr">
+        <is>
+          <t>กรมธรรม์ความรับผิดต่อบุคคลภายนอก</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="n"/>
+      <c r="D18" s="12" t="n"/>
+      <c r="E18" s="12" t="n"/>
+      <c r="F18" s="12" t="n"/>
+      <c r="G18" s="12" t="n"/>
+      <c r="H18" s="12" t="n"/>
+      <c r="I18" s="12" t="n"/>
+      <c r="J18" s="12" t="n"/>
+      <c r="K18" s="12" t="n"/>
+      <c r="L18" s="12">
+        <f>COUNTIF(C18:K18,"?*")-COUNTIF(C18:K18,"Missing")-COUNTIF(C18:K18,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M18" s="12">
+        <f>COUNTIF(C18:K18,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>Alcohol licence (renewed copy)</t>
+        </is>
+      </c>
+      <c r="B19" s="47" t="inlineStr">
+        <is>
+          <t>ใบอนุญาตขายสุราปีนั้น</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="n"/>
+      <c r="D19" s="12" t="n"/>
+      <c r="E19" s="12" t="n"/>
+      <c r="F19" s="12" t="n"/>
+      <c r="G19" s="12" t="n"/>
+      <c r="H19" s="12" t="n"/>
+      <c r="I19" s="12" t="n"/>
+      <c r="J19" s="12" t="n"/>
+      <c r="K19" s="12" t="n"/>
+      <c r="L19" s="12">
+        <f>COUNTIF(C19:K19,"?*")-COUNTIF(C19:K19,"Missing")-COUNTIF(C19:K19,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M19" s="12">
+        <f>COUNTIF(C19:K19,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>Energy conservation audit report</t>
+        </is>
+      </c>
+      <c r="B20" s="47" t="inlineStr">
+        <is>
+          <t>รายงานตรวจสอบการอนุรักษ์พลังงาน</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="n"/>
+      <c r="D20" s="12" t="n"/>
+      <c r="E20" s="12" t="n"/>
+      <c r="F20" s="12" t="n"/>
+      <c r="G20" s="12" t="n"/>
+      <c r="H20" s="12" t="n"/>
+      <c r="I20" s="12" t="n"/>
+      <c r="J20" s="12" t="n"/>
+      <c r="K20" s="12" t="n"/>
+      <c r="L20" s="12">
+        <f>COUNTIF(C20:K20,"?*")-COUNTIF(C20:K20,"Missing")-COUNTIF(C20:K20,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M20" s="12">
+        <f>COUNTIF(C20:K20,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="44" t="inlineStr">
+        <is>
+          <t>2. AES — Ascott Embassy Sathorn Bangkok</t>
+        </is>
+      </c>
+      <c r="B22" s="45" t="n"/>
+      <c r="C22" s="45" t="n"/>
+      <c r="D22" s="45" t="n"/>
+      <c r="E22" s="45" t="n"/>
+      <c r="F22" s="45" t="n"/>
+      <c r="G22" s="45" t="n"/>
+      <c r="H22" s="45" t="n"/>
+      <c r="I22" s="45" t="n"/>
+      <c r="J22" s="45" t="n"/>
+      <c r="K22" s="45" t="n"/>
+      <c r="L22" s="45" t="n"/>
+      <c r="M22" s="45" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="46" t="inlineStr">
+        <is>
+          <t>Document</t>
+        </is>
+      </c>
+      <c r="B23" s="46" t="inlineStr">
+        <is>
+          <t>เอกสาร</t>
+        </is>
+      </c>
+      <c r="C23" s="46" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D23" s="46" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="E23" s="46" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="F23" s="46" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="G23" s="46" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="H23" s="46" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I23" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="J23" s="46" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="K23" s="46" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="L23" s="46" t="inlineStr">
+        <is>
+          <t>Have</t>
+        </is>
+      </c>
+      <c r="M23" s="46" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>EIA monitoring report — 1H</t>
+        </is>
+      </c>
+      <c r="B24" s="47" t="inlineStr">
+        <is>
+          <t>รายงานติดตาม EIA — ครึ่งปีแรก</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="n"/>
+      <c r="D24" s="12" t="n"/>
+      <c r="E24" s="12" t="n"/>
+      <c r="F24" s="12" t="n"/>
+      <c r="G24" s="12" t="n"/>
+      <c r="H24" s="12" t="n"/>
+      <c r="I24" s="12" t="n"/>
+      <c r="J24" s="12" t="n"/>
+      <c r="K24" s="12" t="n"/>
+      <c r="L24" s="12">
+        <f>COUNTIF(C24:K24,"?*")-COUNTIF(C24:K24,"Missing")-COUNTIF(C24:K24,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M24" s="12">
+        <f>COUNTIF(C24:K24,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>EIA monitoring report — 2H</t>
+        </is>
+      </c>
+      <c r="B25" s="47" t="inlineStr">
+        <is>
+          <t>รายงานติดตาม EIA — ครึ่งปีหลัง</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="n"/>
+      <c r="D25" s="12" t="n"/>
+      <c r="E25" s="12" t="n"/>
+      <c r="F25" s="12" t="n"/>
+      <c r="G25" s="12" t="n"/>
+      <c r="H25" s="12" t="n"/>
+      <c r="I25" s="12" t="n"/>
+      <c r="J25" s="12" t="n"/>
+      <c r="K25" s="12" t="n"/>
+      <c r="L25" s="12">
+        <f>COUNTIF(C25:K25,"?*")-COUNTIF(C25:K25,"Missing")-COUNTIF(C25:K25,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M25" s="12">
+        <f>COUNTIF(C25:K25,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>Annual building inspection (Ror.1)</t>
+        </is>
+      </c>
+      <c r="B26" s="47" t="inlineStr">
+        <is>
+          <t>รายงานตรวจสอบอาคาร (ร.1)</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="n"/>
+      <c r="D26" s="12" t="n"/>
+      <c r="E26" s="12" t="n"/>
+      <c r="F26" s="12" t="n"/>
+      <c r="G26" s="12" t="n"/>
+      <c r="H26" s="12" t="n"/>
+      <c r="I26" s="12" t="n"/>
+      <c r="J26" s="12" t="n"/>
+      <c r="K26" s="12" t="n"/>
+      <c r="L26" s="12">
+        <f>COUNTIF(C26:K26,"?*")-COUNTIF(C26:K26,"Missing")-COUNTIF(C26:K26,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M26" s="12">
+        <f>COUNTIF(C26:K26,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Workplace environment assessment</t>
+        </is>
+      </c>
+      <c r="B27" s="47" t="inlineStr">
+        <is>
+          <t>ผลตรวจวัดสภาพแวดล้อมในการทำงาน</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="n"/>
+      <c r="D27" s="12" t="n"/>
+      <c r="E27" s="12" t="n"/>
+      <c r="F27" s="12" t="n"/>
+      <c r="G27" s="12" t="n"/>
+      <c r="H27" s="12" t="n"/>
+      <c r="I27" s="12" t="n"/>
+      <c r="J27" s="12" t="n"/>
+      <c r="K27" s="12" t="n"/>
+      <c r="L27" s="12">
+        <f>COUNTIF(C27:K27,"?*")-COUNTIF(C27:K27,"Missing")-COUNTIF(C27:K27,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M27" s="12">
+        <f>COUNTIF(C27:K27,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>Air / water / wastewater test reports</t>
+        </is>
+      </c>
+      <c r="B28" s="47" t="inlineStr">
+        <is>
+          <t>ผลตรวจอากาศ น้ำ น้ำทิ้ง</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="n"/>
+      <c r="D28" s="12" t="n"/>
+      <c r="E28" s="12" t="n"/>
+      <c r="F28" s="12" t="n"/>
+      <c r="G28" s="12" t="n"/>
+      <c r="H28" s="12" t="n"/>
+      <c r="I28" s="12" t="n"/>
+      <c r="J28" s="12" t="n"/>
+      <c r="K28" s="12" t="n"/>
+      <c r="L28" s="12">
+        <f>COUNTIF(C28:K28,"?*")-COUNTIF(C28:K28,"Missing")-COUNTIF(C28:K28,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M28" s="12">
+        <f>COUNTIF(C28:K28,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>Land &amp; building tax receipt</t>
+        </is>
+      </c>
+      <c r="B29" s="47" t="inlineStr">
+        <is>
+          <t>ใบเสร็จภาษีที่ดินและสิ่งปลูกสร้าง</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="n"/>
+      <c r="D29" s="12" t="n"/>
+      <c r="E29" s="12" t="n"/>
+      <c r="F29" s="12" t="n"/>
+      <c r="G29" s="12" t="n"/>
+      <c r="H29" s="12" t="n"/>
+      <c r="I29" s="12" t="n"/>
+      <c r="J29" s="12" t="n"/>
+      <c r="K29" s="12" t="n"/>
+      <c r="L29" s="12">
+        <f>COUNTIF(C29:K29,"?*")-COUNTIF(C29:K29,"Missing")-COUNTIF(C29:K29,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M29" s="12">
+        <f>COUNTIF(C29:K29,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>Signage tax receipt</t>
+        </is>
+      </c>
+      <c r="B30" s="47" t="inlineStr">
+        <is>
+          <t>ใบเสร็จภาษีป้าย</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="n"/>
+      <c r="D30" s="12" t="n"/>
+      <c r="E30" s="12" t="n"/>
+      <c r="F30" s="12" t="n"/>
+      <c r="G30" s="12" t="n"/>
+      <c r="H30" s="12" t="n"/>
+      <c r="I30" s="12" t="n"/>
+      <c r="J30" s="12" t="n"/>
+      <c r="K30" s="12" t="n"/>
+      <c r="L30" s="12">
+        <f>COUNTIF(C30:K30,"?*")-COUNTIF(C30:K30,"Missing")-COUNTIF(C30:K30,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M30" s="12">
+        <f>COUNTIF(C30:K30,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>Audited FS (EN)</t>
+        </is>
+      </c>
+      <c r="B31" s="47" t="inlineStr">
+        <is>
+          <t>งบการเงินตรวจสอบแล้ว (อังกฤษ)</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="n"/>
+      <c r="D31" s="12" t="n"/>
+      <c r="E31" s="12" t="n"/>
+      <c r="F31" s="12" t="n"/>
+      <c r="G31" s="12" t="n"/>
+      <c r="H31" s="12" t="n"/>
+      <c r="I31" s="12" t="n"/>
+      <c r="J31" s="12" t="n"/>
+      <c r="K31" s="12" t="n"/>
+      <c r="L31" s="12">
+        <f>COUNTIF(C31:K31,"?*")-COUNTIF(C31:K31,"Missing")-COUNTIF(C31:K31,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M31" s="12">
+        <f>COUNTIF(C31:K31,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>Audited FS (TH)</t>
+        </is>
+      </c>
+      <c r="B32" s="47" t="inlineStr">
+        <is>
+          <t>งบการเงินตรวจสอบแล้ว (ไทย)</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="n"/>
+      <c r="D32" s="12" t="n"/>
+      <c r="E32" s="12" t="n"/>
+      <c r="F32" s="12" t="n"/>
+      <c r="G32" s="12" t="n"/>
+      <c r="H32" s="12" t="n"/>
+      <c r="I32" s="12" t="n"/>
+      <c r="J32" s="12" t="n"/>
+      <c r="K32" s="12" t="n"/>
+      <c r="L32" s="12">
+        <f>COUNTIF(C32:K32,"?*")-COUNTIF(C32:K32,"Missing")-COUNTIF(C32:K32,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M32" s="12">
+        <f>COUNTIF(C32:K32,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>PND.50 filing</t>
+        </is>
+      </c>
+      <c r="B33" s="47" t="inlineStr">
+        <is>
+          <t>แบบ ภ.ง.ด.50</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="n"/>
+      <c r="D33" s="12" t="n"/>
+      <c r="E33" s="12" t="n"/>
+      <c r="F33" s="12" t="n"/>
+      <c r="G33" s="12" t="n"/>
+      <c r="H33" s="12" t="n"/>
+      <c r="I33" s="12" t="n"/>
+      <c r="J33" s="12" t="n"/>
+      <c r="K33" s="12" t="n"/>
+      <c r="L33" s="12">
+        <f>COUNTIF(C33:K33,"?*")-COUNTIF(C33:K33,"Missing")-COUNTIF(C33:K33,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M33" s="12">
+        <f>COUNTIF(C33:K33,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>PND.51 filing</t>
+        </is>
+      </c>
+      <c r="B34" s="47" t="inlineStr">
+        <is>
+          <t>แบบ ภ.ง.ด.51</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="n"/>
+      <c r="D34" s="12" t="n"/>
+      <c r="E34" s="12" t="n"/>
+      <c r="F34" s="12" t="n"/>
+      <c r="G34" s="12" t="n"/>
+      <c r="H34" s="12" t="n"/>
+      <c r="I34" s="12" t="n"/>
+      <c r="J34" s="12" t="n"/>
+      <c r="K34" s="12" t="n"/>
+      <c r="L34" s="12">
+        <f>COUNTIF(C34:K34,"?*")-COUNTIF(C34:K34,"Missing")-COUNTIF(C34:K34,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M34" s="12">
+        <f>COUNTIF(C34:K34,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>Insurance policy set (IAR / BI / PV)</t>
+        </is>
+      </c>
+      <c r="B35" s="47" t="inlineStr">
+        <is>
+          <t>กรมธรรม์ประกันทรัพย์สินชุดปี</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="n"/>
+      <c r="D35" s="12" t="n"/>
+      <c r="E35" s="12" t="n"/>
+      <c r="F35" s="12" t="n"/>
+      <c r="G35" s="12" t="n"/>
+      <c r="H35" s="12" t="n"/>
+      <c r="I35" s="12" t="n"/>
+      <c r="J35" s="12" t="n"/>
+      <c r="K35" s="12" t="n"/>
+      <c r="L35" s="12">
+        <f>COUNTIF(C35:K35,"?*")-COUNTIF(C35:K35,"Missing")-COUNTIF(C35:K35,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M35" s="12">
+        <f>COUNTIF(C35:K35,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>Public liability policy</t>
+        </is>
+      </c>
+      <c r="B36" s="47" t="inlineStr">
+        <is>
+          <t>กรมธรรม์ความรับผิดต่อบุคคลภายนอก</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="n"/>
+      <c r="D36" s="12" t="n"/>
+      <c r="E36" s="12" t="n"/>
+      <c r="F36" s="12" t="n"/>
+      <c r="G36" s="12" t="n"/>
+      <c r="H36" s="12" t="n"/>
+      <c r="I36" s="12" t="n"/>
+      <c r="J36" s="12" t="n"/>
+      <c r="K36" s="12" t="n"/>
+      <c r="L36" s="12">
+        <f>COUNTIF(C36:K36,"?*")-COUNTIF(C36:K36,"Missing")-COUNTIF(C36:K36,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M36" s="12">
+        <f>COUNTIF(C36:K36,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>Alcohol licence (renewed copy)</t>
+        </is>
+      </c>
+      <c r="B37" s="47" t="inlineStr">
+        <is>
+          <t>ใบอนุญาตขายสุราปีนั้น</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="n"/>
+      <c r="D37" s="12" t="n"/>
+      <c r="E37" s="12" t="n"/>
+      <c r="F37" s="12" t="n"/>
+      <c r="G37" s="12" t="n"/>
+      <c r="H37" s="12" t="n"/>
+      <c r="I37" s="12" t="n"/>
+      <c r="J37" s="12" t="n"/>
+      <c r="K37" s="12" t="n"/>
+      <c r="L37" s="12">
+        <f>COUNTIF(C37:K37,"?*")-COUNTIF(C37:K37,"Missing")-COUNTIF(C37:K37,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M37" s="12">
+        <f>COUNTIF(C37:K37,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>Energy conservation audit report</t>
+        </is>
+      </c>
+      <c r="B38" s="47" t="inlineStr">
+        <is>
+          <t>รายงานตรวจสอบการอนุรักษ์พลังงาน</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="n"/>
+      <c r="D38" s="12" t="n"/>
+      <c r="E38" s="12" t="n"/>
+      <c r="F38" s="12" t="n"/>
+      <c r="G38" s="12" t="n"/>
+      <c r="H38" s="12" t="n"/>
+      <c r="I38" s="12" t="n"/>
+      <c r="J38" s="12" t="n"/>
+      <c r="K38" s="12" t="n"/>
+      <c r="L38" s="12">
+        <f>COUNTIF(C38:K38,"?*")-COUNTIF(C38:K38,"Missing")-COUNTIF(C38:K38,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M38" s="12">
+        <f>COUNTIF(C38:K38,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="44" t="inlineStr">
+        <is>
+          <t>3. LYF — lyf Sukhumvit 8 Bangkok</t>
+        </is>
+      </c>
+      <c r="B40" s="45" t="n"/>
+      <c r="C40" s="45" t="n"/>
+      <c r="D40" s="45" t="n"/>
+      <c r="E40" s="45" t="n"/>
+      <c r="F40" s="45" t="n"/>
+      <c r="G40" s="45" t="n"/>
+      <c r="H40" s="45" t="n"/>
+      <c r="I40" s="45" t="n"/>
+      <c r="J40" s="45" t="n"/>
+      <c r="K40" s="45" t="n"/>
+      <c r="L40" s="45" t="n"/>
+      <c r="M40" s="45" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="46" t="inlineStr">
+        <is>
+          <t>Document</t>
+        </is>
+      </c>
+      <c r="B41" s="46" t="inlineStr">
+        <is>
+          <t>เอกสาร</t>
+        </is>
+      </c>
+      <c r="C41" s="46" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D41" s="46" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="E41" s="46" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="F41" s="46" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="G41" s="46" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="H41" s="46" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I41" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="J41" s="46" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="K41" s="46" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="L41" s="46" t="inlineStr">
+        <is>
+          <t>Have</t>
+        </is>
+      </c>
+      <c r="M41" s="46" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>EIA monitoring report — 1H</t>
+        </is>
+      </c>
+      <c r="B42" s="47" t="inlineStr">
+        <is>
+          <t>รายงานติดตาม EIA — ครึ่งปีแรก</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="n"/>
+      <c r="D42" s="12" t="n"/>
+      <c r="E42" s="12" t="n"/>
+      <c r="F42" s="12" t="n"/>
+      <c r="G42" s="12" t="n"/>
+      <c r="H42" s="12" t="n"/>
+      <c r="I42" s="12" t="n"/>
+      <c r="J42" s="12" t="n"/>
+      <c r="K42" s="12" t="n"/>
+      <c r="L42" s="12">
+        <f>COUNTIF(C42:K42,"?*")-COUNTIF(C42:K42,"Missing")-COUNTIF(C42:K42,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M42" s="12">
+        <f>COUNTIF(C42:K42,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="11" t="inlineStr">
+        <is>
+          <t>EIA monitoring report — 2H</t>
+        </is>
+      </c>
+      <c r="B43" s="47" t="inlineStr">
+        <is>
+          <t>รายงานติดตาม EIA — ครึ่งปีหลัง</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="n"/>
+      <c r="D43" s="12" t="n"/>
+      <c r="E43" s="12" t="n"/>
+      <c r="F43" s="12" t="n"/>
+      <c r="G43" s="12" t="n"/>
+      <c r="H43" s="12" t="n"/>
+      <c r="I43" s="12" t="n"/>
+      <c r="J43" s="12" t="n"/>
+      <c r="K43" s="12" t="n"/>
+      <c r="L43" s="12">
+        <f>COUNTIF(C43:K43,"?*")-COUNTIF(C43:K43,"Missing")-COUNTIF(C43:K43,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M43" s="12">
+        <f>COUNTIF(C43:K43,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="11" t="inlineStr">
+        <is>
+          <t>Annual building inspection (Ror.1)</t>
+        </is>
+      </c>
+      <c r="B44" s="47" t="inlineStr">
+        <is>
+          <t>รายงานตรวจสอบอาคาร (ร.1)</t>
+        </is>
+      </c>
+      <c r="C44" s="12" t="n"/>
+      <c r="D44" s="12" t="n"/>
+      <c r="E44" s="12" t="n"/>
+      <c r="F44" s="12" t="n"/>
+      <c r="G44" s="12" t="n"/>
+      <c r="H44" s="12" t="n"/>
+      <c r="I44" s="12" t="n"/>
+      <c r="J44" s="12" t="n"/>
+      <c r="K44" s="12" t="n"/>
+      <c r="L44" s="12">
+        <f>COUNTIF(C44:K44,"?*")-COUNTIF(C44:K44,"Missing")-COUNTIF(C44:K44,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M44" s="12">
+        <f>COUNTIF(C44:K44,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="11" t="inlineStr">
+        <is>
+          <t>Workplace environment assessment</t>
+        </is>
+      </c>
+      <c r="B45" s="47" t="inlineStr">
+        <is>
+          <t>ผลตรวจวัดสภาพแวดล้อมในการทำงาน</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="n"/>
+      <c r="D45" s="12" t="n"/>
+      <c r="E45" s="12" t="n"/>
+      <c r="F45" s="12" t="n"/>
+      <c r="G45" s="12" t="n"/>
+      <c r="H45" s="12" t="n"/>
+      <c r="I45" s="12" t="n"/>
+      <c r="J45" s="12" t="n"/>
+      <c r="K45" s="12" t="n"/>
+      <c r="L45" s="12">
+        <f>COUNTIF(C45:K45,"?*")-COUNTIF(C45:K45,"Missing")-COUNTIF(C45:K45,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M45" s="12">
+        <f>COUNTIF(C45:K45,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>Air / water / wastewater test reports</t>
+        </is>
+      </c>
+      <c r="B46" s="47" t="inlineStr">
+        <is>
+          <t>ผลตรวจอากาศ น้ำ น้ำทิ้ง</t>
+        </is>
+      </c>
+      <c r="C46" s="12" t="n"/>
+      <c r="D46" s="12" t="n"/>
+      <c r="E46" s="12" t="n"/>
+      <c r="F46" s="12" t="n"/>
+      <c r="G46" s="12" t="n"/>
+      <c r="H46" s="12" t="n"/>
+      <c r="I46" s="12" t="n"/>
+      <c r="J46" s="12" t="n"/>
+      <c r="K46" s="12" t="n"/>
+      <c r="L46" s="12">
+        <f>COUNTIF(C46:K46,"?*")-COUNTIF(C46:K46,"Missing")-COUNTIF(C46:K46,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M46" s="12">
+        <f>COUNTIF(C46:K46,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t>Land &amp; building tax receipt</t>
+        </is>
+      </c>
+      <c r="B47" s="47" t="inlineStr">
+        <is>
+          <t>ใบเสร็จภาษีที่ดินและสิ่งปลูกสร้าง</t>
+        </is>
+      </c>
+      <c r="C47" s="12" t="n"/>
+      <c r="D47" s="12" t="n"/>
+      <c r="E47" s="12" t="n"/>
+      <c r="F47" s="12" t="n"/>
+      <c r="G47" s="12" t="n"/>
+      <c r="H47" s="12" t="n"/>
+      <c r="I47" s="12" t="n"/>
+      <c r="J47" s="12" t="n"/>
+      <c r="K47" s="12" t="n"/>
+      <c r="L47" s="12">
+        <f>COUNTIF(C47:K47,"?*")-COUNTIF(C47:K47,"Missing")-COUNTIF(C47:K47,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M47" s="12">
+        <f>COUNTIF(C47:K47,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="11" t="inlineStr">
+        <is>
+          <t>Signage tax receipt</t>
+        </is>
+      </c>
+      <c r="B48" s="47" t="inlineStr">
+        <is>
+          <t>ใบเสร็จภาษีป้าย</t>
+        </is>
+      </c>
+      <c r="C48" s="12" t="n"/>
+      <c r="D48" s="12" t="n"/>
+      <c r="E48" s="12" t="n"/>
+      <c r="F48" s="12" t="n"/>
+      <c r="G48" s="12" t="n"/>
+      <c r="H48" s="12" t="n"/>
+      <c r="I48" s="12" t="n"/>
+      <c r="J48" s="12" t="n"/>
+      <c r="K48" s="12" t="n"/>
+      <c r="L48" s="12">
+        <f>COUNTIF(C48:K48,"?*")-COUNTIF(C48:K48,"Missing")-COUNTIF(C48:K48,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M48" s="12">
+        <f>COUNTIF(C48:K48,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="11" t="inlineStr">
+        <is>
+          <t>Audited FS (EN)</t>
+        </is>
+      </c>
+      <c r="B49" s="47" t="inlineStr">
+        <is>
+          <t>งบการเงินตรวจสอบแล้ว (อังกฤษ)</t>
+        </is>
+      </c>
+      <c r="C49" s="12" t="n"/>
+      <c r="D49" s="12" t="n"/>
+      <c r="E49" s="12" t="n"/>
+      <c r="F49" s="12" t="n"/>
+      <c r="G49" s="12" t="n"/>
+      <c r="H49" s="12" t="n"/>
+      <c r="I49" s="12" t="n"/>
+      <c r="J49" s="12" t="n"/>
+      <c r="K49" s="12" t="n"/>
+      <c r="L49" s="12">
+        <f>COUNTIF(C49:K49,"?*")-COUNTIF(C49:K49,"Missing")-COUNTIF(C49:K49,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M49" s="12">
+        <f>COUNTIF(C49:K49,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="11" t="inlineStr">
+        <is>
+          <t>Audited FS (TH)</t>
+        </is>
+      </c>
+      <c r="B50" s="47" t="inlineStr">
+        <is>
+          <t>งบการเงินตรวจสอบแล้ว (ไทย)</t>
+        </is>
+      </c>
+      <c r="C50" s="12" t="n"/>
+      <c r="D50" s="12" t="n"/>
+      <c r="E50" s="12" t="n"/>
+      <c r="F50" s="12" t="n"/>
+      <c r="G50" s="12" t="n"/>
+      <c r="H50" s="12" t="n"/>
+      <c r="I50" s="12" t="n"/>
+      <c r="J50" s="12" t="n"/>
+      <c r="K50" s="12" t="n"/>
+      <c r="L50" s="12">
+        <f>COUNTIF(C50:K50,"?*")-COUNTIF(C50:K50,"Missing")-COUNTIF(C50:K50,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M50" s="12">
+        <f>COUNTIF(C50:K50,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>PND.50 filing</t>
+        </is>
+      </c>
+      <c r="B51" s="47" t="inlineStr">
+        <is>
+          <t>แบบ ภ.ง.ด.50</t>
+        </is>
+      </c>
+      <c r="C51" s="12" t="n"/>
+      <c r="D51" s="12" t="n"/>
+      <c r="E51" s="12" t="n"/>
+      <c r="F51" s="12" t="n"/>
+      <c r="G51" s="12" t="n"/>
+      <c r="H51" s="12" t="n"/>
+      <c r="I51" s="12" t="n"/>
+      <c r="J51" s="12" t="n"/>
+      <c r="K51" s="12" t="n"/>
+      <c r="L51" s="12">
+        <f>COUNTIF(C51:K51,"?*")-COUNTIF(C51:K51,"Missing")-COUNTIF(C51:K51,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M51" s="12">
+        <f>COUNTIF(C51:K51,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="11" t="inlineStr">
+        <is>
+          <t>PND.51 filing</t>
+        </is>
+      </c>
+      <c r="B52" s="47" t="inlineStr">
+        <is>
+          <t>แบบ ภ.ง.ด.51</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="n"/>
+      <c r="D52" s="12" t="n"/>
+      <c r="E52" s="12" t="n"/>
+      <c r="F52" s="12" t="n"/>
+      <c r="G52" s="12" t="n"/>
+      <c r="H52" s="12" t="n"/>
+      <c r="I52" s="12" t="n"/>
+      <c r="J52" s="12" t="n"/>
+      <c r="K52" s="12" t="n"/>
+      <c r="L52" s="12">
+        <f>COUNTIF(C52:K52,"?*")-COUNTIF(C52:K52,"Missing")-COUNTIF(C52:K52,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M52" s="12">
+        <f>COUNTIF(C52:K52,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="11" t="inlineStr">
+        <is>
+          <t>Insurance policy set (IAR / BI / PV)</t>
+        </is>
+      </c>
+      <c r="B53" s="47" t="inlineStr">
+        <is>
+          <t>กรมธรรม์ประกันทรัพย์สินชุดปี</t>
+        </is>
+      </c>
+      <c r="C53" s="12" t="n"/>
+      <c r="D53" s="12" t="n"/>
+      <c r="E53" s="12" t="n"/>
+      <c r="F53" s="12" t="n"/>
+      <c r="G53" s="12" t="n"/>
+      <c r="H53" s="12" t="n"/>
+      <c r="I53" s="12" t="n"/>
+      <c r="J53" s="12" t="n"/>
+      <c r="K53" s="12" t="n"/>
+      <c r="L53" s="12">
+        <f>COUNTIF(C53:K53,"?*")-COUNTIF(C53:K53,"Missing")-COUNTIF(C53:K53,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M53" s="12">
+        <f>COUNTIF(C53:K53,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="11" t="inlineStr">
+        <is>
+          <t>Public liability policy</t>
+        </is>
+      </c>
+      <c r="B54" s="47" t="inlineStr">
+        <is>
+          <t>กรมธรรม์ความรับผิดต่อบุคคลภายนอก</t>
+        </is>
+      </c>
+      <c r="C54" s="12" t="n"/>
+      <c r="D54" s="12" t="n"/>
+      <c r="E54" s="12" t="n"/>
+      <c r="F54" s="12" t="n"/>
+      <c r="G54" s="12" t="n"/>
+      <c r="H54" s="12" t="n"/>
+      <c r="I54" s="12" t="n"/>
+      <c r="J54" s="12" t="n"/>
+      <c r="K54" s="12" t="n"/>
+      <c r="L54" s="12">
+        <f>COUNTIF(C54:K54,"?*")-COUNTIF(C54:K54,"Missing")-COUNTIF(C54:K54,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M54" s="12">
+        <f>COUNTIF(C54:K54,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="11" t="inlineStr">
+        <is>
+          <t>Alcohol licence (renewed copy)</t>
+        </is>
+      </c>
+      <c r="B55" s="47" t="inlineStr">
+        <is>
+          <t>ใบอนุญาตขายสุราปีนั้น</t>
+        </is>
+      </c>
+      <c r="C55" s="12" t="n"/>
+      <c r="D55" s="12" t="n"/>
+      <c r="E55" s="12" t="n"/>
+      <c r="F55" s="12" t="n"/>
+      <c r="G55" s="12" t="n"/>
+      <c r="H55" s="12" t="n"/>
+      <c r="I55" s="12" t="n"/>
+      <c r="J55" s="12" t="n"/>
+      <c r="K55" s="12" t="n"/>
+      <c r="L55" s="12">
+        <f>COUNTIF(C55:K55,"?*")-COUNTIF(C55:K55,"Missing")-COUNTIF(C55:K55,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M55" s="12">
+        <f>COUNTIF(C55:K55,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="11" t="inlineStr">
+        <is>
+          <t>Energy conservation audit report</t>
+        </is>
+      </c>
+      <c r="B56" s="47" t="inlineStr">
+        <is>
+          <t>รายงานตรวจสอบการอนุรักษ์พลังงาน</t>
+        </is>
+      </c>
+      <c r="C56" s="12" t="n"/>
+      <c r="D56" s="12" t="n"/>
+      <c r="E56" s="12" t="n"/>
+      <c r="F56" s="12" t="n"/>
+      <c r="G56" s="12" t="n"/>
+      <c r="H56" s="12" t="n"/>
+      <c r="I56" s="12" t="n"/>
+      <c r="J56" s="12" t="n"/>
+      <c r="K56" s="12" t="n"/>
+      <c r="L56" s="12">
+        <f>COUNTIF(C56:K56,"?*")-COUNTIF(C56:K56,"Missing")-COUNTIF(C56:K56,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M56" s="12">
+        <f>COUNTIF(C56:K56,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="44" t="inlineStr">
+        <is>
+          <t>4. SP — Somerset Pattaya</t>
+        </is>
+      </c>
+      <c r="B58" s="45" t="n"/>
+      <c r="C58" s="45" t="n"/>
+      <c r="D58" s="45" t="n"/>
+      <c r="E58" s="45" t="n"/>
+      <c r="F58" s="45" t="n"/>
+      <c r="G58" s="45" t="n"/>
+      <c r="H58" s="45" t="n"/>
+      <c r="I58" s="45" t="n"/>
+      <c r="J58" s="45" t="n"/>
+      <c r="K58" s="45" t="n"/>
+      <c r="L58" s="45" t="n"/>
+      <c r="M58" s="45" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="46" t="inlineStr">
+        <is>
+          <t>Document</t>
+        </is>
+      </c>
+      <c r="B59" s="46" t="inlineStr">
+        <is>
+          <t>เอกสาร</t>
+        </is>
+      </c>
+      <c r="C59" s="46" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D59" s="46" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="E59" s="46" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="F59" s="46" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="G59" s="46" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="H59" s="46" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I59" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="J59" s="46" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="K59" s="46" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="L59" s="46" t="inlineStr">
+        <is>
+          <t>Have</t>
+        </is>
+      </c>
+      <c r="M59" s="46" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t>EIA monitoring report — 1H</t>
+        </is>
+      </c>
+      <c r="B60" s="47" t="inlineStr">
+        <is>
+          <t>รายงานติดตาม EIA — ครึ่งปีแรก</t>
+        </is>
+      </c>
+      <c r="C60" s="12" t="n"/>
+      <c r="D60" s="12" t="n"/>
+      <c r="E60" s="12" t="n"/>
+      <c r="F60" s="12" t="n"/>
+      <c r="G60" s="12" t="n"/>
+      <c r="H60" s="12" t="n"/>
+      <c r="I60" s="12" t="n"/>
+      <c r="J60" s="12" t="n"/>
+      <c r="K60" s="12" t="n"/>
+      <c r="L60" s="12">
+        <f>COUNTIF(C60:K60,"?*")-COUNTIF(C60:K60,"Missing")-COUNTIF(C60:K60,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M60" s="12">
+        <f>COUNTIF(C60:K60,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="11" t="inlineStr">
+        <is>
+          <t>EIA monitoring report — 2H</t>
+        </is>
+      </c>
+      <c r="B61" s="47" t="inlineStr">
+        <is>
+          <t>รายงานติดตาม EIA — ครึ่งปีหลัง</t>
+        </is>
+      </c>
+      <c r="C61" s="12" t="n"/>
+      <c r="D61" s="12" t="n"/>
+      <c r="E61" s="12" t="n"/>
+      <c r="F61" s="12" t="n"/>
+      <c r="G61" s="12" t="n"/>
+      <c r="H61" s="12" t="n"/>
+      <c r="I61" s="12" t="n"/>
+      <c r="J61" s="12" t="n"/>
+      <c r="K61" s="12" t="n"/>
+      <c r="L61" s="12">
+        <f>COUNTIF(C61:K61,"?*")-COUNTIF(C61:K61,"Missing")-COUNTIF(C61:K61,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M61" s="12">
+        <f>COUNTIF(C61:K61,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
+          <t>Annual building inspection (Ror.1)</t>
+        </is>
+      </c>
+      <c r="B62" s="47" t="inlineStr">
+        <is>
+          <t>รายงานตรวจสอบอาคาร (ร.1)</t>
+        </is>
+      </c>
+      <c r="C62" s="12" t="n"/>
+      <c r="D62" s="12" t="n"/>
+      <c r="E62" s="12" t="n"/>
+      <c r="F62" s="12" t="n"/>
+      <c r="G62" s="12" t="n"/>
+      <c r="H62" s="12" t="n"/>
+      <c r="I62" s="12" t="n"/>
+      <c r="J62" s="12" t="n"/>
+      <c r="K62" s="12" t="n"/>
+      <c r="L62" s="12">
+        <f>COUNTIF(C62:K62,"?*")-COUNTIF(C62:K62,"Missing")-COUNTIF(C62:K62,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M62" s="12">
+        <f>COUNTIF(C62:K62,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="11" t="inlineStr">
+        <is>
+          <t>Workplace environment assessment</t>
+        </is>
+      </c>
+      <c r="B63" s="47" t="inlineStr">
+        <is>
+          <t>ผลตรวจวัดสภาพแวดล้อมในการทำงาน</t>
+        </is>
+      </c>
+      <c r="C63" s="12" t="n"/>
+      <c r="D63" s="12" t="n"/>
+      <c r="E63" s="12" t="n"/>
+      <c r="F63" s="12" t="n"/>
+      <c r="G63" s="12" t="n"/>
+      <c r="H63" s="12" t="n"/>
+      <c r="I63" s="12" t="n"/>
+      <c r="J63" s="12" t="n"/>
+      <c r="K63" s="12" t="n"/>
+      <c r="L63" s="12">
+        <f>COUNTIF(C63:K63,"?*")-COUNTIF(C63:K63,"Missing")-COUNTIF(C63:K63,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M63" s="12">
+        <f>COUNTIF(C63:K63,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="inlineStr">
+        <is>
+          <t>Air / water / wastewater test reports</t>
+        </is>
+      </c>
+      <c r="B64" s="47" t="inlineStr">
+        <is>
+          <t>ผลตรวจอากาศ น้ำ น้ำทิ้ง</t>
+        </is>
+      </c>
+      <c r="C64" s="12" t="n"/>
+      <c r="D64" s="12" t="n"/>
+      <c r="E64" s="12" t="n"/>
+      <c r="F64" s="12" t="n"/>
+      <c r="G64" s="12" t="n"/>
+      <c r="H64" s="12" t="n"/>
+      <c r="I64" s="12" t="n"/>
+      <c r="J64" s="12" t="n"/>
+      <c r="K64" s="12" t="n"/>
+      <c r="L64" s="12">
+        <f>COUNTIF(C64:K64,"?*")-COUNTIF(C64:K64,"Missing")-COUNTIF(C64:K64,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M64" s="12">
+        <f>COUNTIF(C64:K64,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="11" t="inlineStr">
+        <is>
+          <t>Land &amp; building tax receipt</t>
+        </is>
+      </c>
+      <c r="B65" s="47" t="inlineStr">
+        <is>
+          <t>ใบเสร็จภาษีที่ดินและสิ่งปลูกสร้าง</t>
+        </is>
+      </c>
+      <c r="C65" s="12" t="n"/>
+      <c r="D65" s="12" t="n"/>
+      <c r="E65" s="12" t="n"/>
+      <c r="F65" s="12" t="n"/>
+      <c r="G65" s="12" t="n"/>
+      <c r="H65" s="12" t="n"/>
+      <c r="I65" s="12" t="n"/>
+      <c r="J65" s="12" t="n"/>
+      <c r="K65" s="12" t="n"/>
+      <c r="L65" s="12">
+        <f>COUNTIF(C65:K65,"?*")-COUNTIF(C65:K65,"Missing")-COUNTIF(C65:K65,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M65" s="12">
+        <f>COUNTIF(C65:K65,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="inlineStr">
+        <is>
+          <t>Signage tax receipt</t>
+        </is>
+      </c>
+      <c r="B66" s="47" t="inlineStr">
+        <is>
+          <t>ใบเสร็จภาษีป้าย</t>
+        </is>
+      </c>
+      <c r="C66" s="12" t="n"/>
+      <c r="D66" s="12" t="n"/>
+      <c r="E66" s="12" t="n"/>
+      <c r="F66" s="12" t="n"/>
+      <c r="G66" s="12" t="n"/>
+      <c r="H66" s="12" t="n"/>
+      <c r="I66" s="12" t="n"/>
+      <c r="J66" s="12" t="n"/>
+      <c r="K66" s="12" t="n"/>
+      <c r="L66" s="12">
+        <f>COUNTIF(C66:K66,"?*")-COUNTIF(C66:K66,"Missing")-COUNTIF(C66:K66,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M66" s="12">
+        <f>COUNTIF(C66:K66,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="11" t="inlineStr">
+        <is>
+          <t>Audited FS (EN)</t>
+        </is>
+      </c>
+      <c r="B67" s="47" t="inlineStr">
+        <is>
+          <t>งบการเงินตรวจสอบแล้ว (อังกฤษ)</t>
+        </is>
+      </c>
+      <c r="C67" s="12" t="n"/>
+      <c r="D67" s="12" t="n"/>
+      <c r="E67" s="12" t="n"/>
+      <c r="F67" s="12" t="n"/>
+      <c r="G67" s="12" t="n"/>
+      <c r="H67" s="12" t="n"/>
+      <c r="I67" s="12" t="n"/>
+      <c r="J67" s="12" t="n"/>
+      <c r="K67" s="12" t="n"/>
+      <c r="L67" s="12">
+        <f>COUNTIF(C67:K67,"?*")-COUNTIF(C67:K67,"Missing")-COUNTIF(C67:K67,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M67" s="12">
+        <f>COUNTIF(C67:K67,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="inlineStr">
+        <is>
+          <t>Audited FS (TH)</t>
+        </is>
+      </c>
+      <c r="B68" s="47" t="inlineStr">
+        <is>
+          <t>งบการเงินตรวจสอบแล้ว (ไทย)</t>
+        </is>
+      </c>
+      <c r="C68" s="12" t="n"/>
+      <c r="D68" s="12" t="n"/>
+      <c r="E68" s="12" t="n"/>
+      <c r="F68" s="12" t="n"/>
+      <c r="G68" s="12" t="n"/>
+      <c r="H68" s="12" t="n"/>
+      <c r="I68" s="12" t="n"/>
+      <c r="J68" s="12" t="n"/>
+      <c r="K68" s="12" t="n"/>
+      <c r="L68" s="12">
+        <f>COUNTIF(C68:K68,"?*")-COUNTIF(C68:K68,"Missing")-COUNTIF(C68:K68,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M68" s="12">
+        <f>COUNTIF(C68:K68,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="11" t="inlineStr">
+        <is>
+          <t>PND.50 filing</t>
+        </is>
+      </c>
+      <c r="B69" s="47" t="inlineStr">
+        <is>
+          <t>แบบ ภ.ง.ด.50</t>
+        </is>
+      </c>
+      <c r="C69" s="12" t="n"/>
+      <c r="D69" s="12" t="n"/>
+      <c r="E69" s="12" t="n"/>
+      <c r="F69" s="12" t="n"/>
+      <c r="G69" s="12" t="n"/>
+      <c r="H69" s="12" t="n"/>
+      <c r="I69" s="12" t="n"/>
+      <c r="J69" s="12" t="n"/>
+      <c r="K69" s="12" t="n"/>
+      <c r="L69" s="12">
+        <f>COUNTIF(C69:K69,"?*")-COUNTIF(C69:K69,"Missing")-COUNTIF(C69:K69,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M69" s="12">
+        <f>COUNTIF(C69:K69,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="inlineStr">
+        <is>
+          <t>PND.51 filing</t>
+        </is>
+      </c>
+      <c r="B70" s="47" t="inlineStr">
+        <is>
+          <t>แบบ ภ.ง.ด.51</t>
+        </is>
+      </c>
+      <c r="C70" s="12" t="n"/>
+      <c r="D70" s="12" t="n"/>
+      <c r="E70" s="12" t="n"/>
+      <c r="F70" s="12" t="n"/>
+      <c r="G70" s="12" t="n"/>
+      <c r="H70" s="12" t="n"/>
+      <c r="I70" s="12" t="n"/>
+      <c r="J70" s="12" t="n"/>
+      <c r="K70" s="12" t="n"/>
+      <c r="L70" s="12">
+        <f>COUNTIF(C70:K70,"?*")-COUNTIF(C70:K70,"Missing")-COUNTIF(C70:K70,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M70" s="12">
+        <f>COUNTIF(C70:K70,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="11" t="inlineStr">
+        <is>
+          <t>Insurance policy set (IAR / BI / PV)</t>
+        </is>
+      </c>
+      <c r="B71" s="47" t="inlineStr">
+        <is>
+          <t>กรมธรรม์ประกันทรัพย์สินชุดปี</t>
+        </is>
+      </c>
+      <c r="C71" s="12" t="n"/>
+      <c r="D71" s="12" t="n"/>
+      <c r="E71" s="12" t="n"/>
+      <c r="F71" s="12" t="n"/>
+      <c r="G71" s="12" t="n"/>
+      <c r="H71" s="12" t="n"/>
+      <c r="I71" s="12" t="n"/>
+      <c r="J71" s="12" t="n"/>
+      <c r="K71" s="12" t="n"/>
+      <c r="L71" s="12">
+        <f>COUNTIF(C71:K71,"?*")-COUNTIF(C71:K71,"Missing")-COUNTIF(C71:K71,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M71" s="12">
+        <f>COUNTIF(C71:K71,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="inlineStr">
+        <is>
+          <t>Public liability policy</t>
+        </is>
+      </c>
+      <c r="B72" s="47" t="inlineStr">
+        <is>
+          <t>กรมธรรม์ความรับผิดต่อบุคคลภายนอก</t>
+        </is>
+      </c>
+      <c r="C72" s="12" t="n"/>
+      <c r="D72" s="12" t="n"/>
+      <c r="E72" s="12" t="n"/>
+      <c r="F72" s="12" t="n"/>
+      <c r="G72" s="12" t="n"/>
+      <c r="H72" s="12" t="n"/>
+      <c r="I72" s="12" t="n"/>
+      <c r="J72" s="12" t="n"/>
+      <c r="K72" s="12" t="n"/>
+      <c r="L72" s="12">
+        <f>COUNTIF(C72:K72,"?*")-COUNTIF(C72:K72,"Missing")-COUNTIF(C72:K72,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M72" s="12">
+        <f>COUNTIF(C72:K72,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="11" t="inlineStr">
+        <is>
+          <t>Alcohol licence (renewed copy)</t>
+        </is>
+      </c>
+      <c r="B73" s="47" t="inlineStr">
+        <is>
+          <t>ใบอนุญาตขายสุราปีนั้น</t>
+        </is>
+      </c>
+      <c r="C73" s="12" t="n"/>
+      <c r="D73" s="12" t="n"/>
+      <c r="E73" s="12" t="n"/>
+      <c r="F73" s="12" t="n"/>
+      <c r="G73" s="12" t="n"/>
+      <c r="H73" s="12" t="n"/>
+      <c r="I73" s="12" t="n"/>
+      <c r="J73" s="12" t="n"/>
+      <c r="K73" s="12" t="n"/>
+      <c r="L73" s="12">
+        <f>COUNTIF(C73:K73,"?*")-COUNTIF(C73:K73,"Missing")-COUNTIF(C73:K73,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M73" s="12">
+        <f>COUNTIF(C73:K73,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="11" t="inlineStr">
+        <is>
+          <t>Energy conservation audit report</t>
+        </is>
+      </c>
+      <c r="B74" s="47" t="inlineStr">
+        <is>
+          <t>รายงานตรวจสอบการอนุรักษ์พลังงาน</t>
+        </is>
+      </c>
+      <c r="C74" s="12" t="n"/>
+      <c r="D74" s="12" t="n"/>
+      <c r="E74" s="12" t="n"/>
+      <c r="F74" s="12" t="n"/>
+      <c r="G74" s="12" t="n"/>
+      <c r="H74" s="12" t="n"/>
+      <c r="I74" s="12" t="n"/>
+      <c r="J74" s="12" t="n"/>
+      <c r="K74" s="12" t="n"/>
+      <c r="L74" s="12">
+        <f>COUNTIF(C74:K74,"?*")-COUNTIF(C74:K74,"Missing")-COUNTIF(C74:K74,"N/A")</f>
+        <v/>
+      </c>
+      <c r="M74" s="12">
+        <f>COUNTIF(C74:K74,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C6:K20">
+    <cfRule type="expression" priority="1" dxfId="1" stopIfTrue="1">
+      <formula>C6="Missing"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="6" stopIfTrue="1">
+      <formula>C6="N/A"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="3" stopIfTrue="1">
+      <formula>C6&lt;&gt;""</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="7" stopIfTrue="1">
+      <formula>C6=""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M6:M20">
+    <cfRule type="expression" priority="5" dxfId="1">
+      <formula>M6&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L6:L20">
+    <cfRule type="expression" priority="6" dxfId="3">
+      <formula>L6&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C24:K38">
+    <cfRule type="expression" priority="7" dxfId="1" stopIfTrue="1">
+      <formula>C24="Missing"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="6" stopIfTrue="1">
+      <formula>C24="N/A"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" dxfId="3" stopIfTrue="1">
+      <formula>C24&lt;&gt;""</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="7" stopIfTrue="1">
+      <formula>C24=""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M24:M38">
+    <cfRule type="expression" priority="11" dxfId="1">
+      <formula>M24&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L24:L38">
+    <cfRule type="expression" priority="12" dxfId="3">
+      <formula>L24&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C42:K56">
+    <cfRule type="expression" priority="13" dxfId="1" stopIfTrue="1">
+      <formula>C42="Missing"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="6" stopIfTrue="1">
+      <formula>C42="N/A"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" dxfId="3" stopIfTrue="1">
+      <formula>C42&lt;&gt;""</formula>
+    </cfRule>
+    <cfRule type="expression" priority="16" dxfId="7" stopIfTrue="1">
+      <formula>C42=""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M42:M56">
+    <cfRule type="expression" priority="17" dxfId="1">
+      <formula>M42&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L42:L56">
+    <cfRule type="expression" priority="18" dxfId="3">
+      <formula>L42&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C60:K74">
+    <cfRule type="expression" priority="19" dxfId="1" stopIfTrue="1">
+      <formula>C60="Missing"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="20" dxfId="6" stopIfTrue="1">
+      <formula>C60="N/A"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="21" dxfId="3" stopIfTrue="1">
+      <formula>C60&lt;&gt;""</formula>
+    </cfRule>
+    <cfRule type="expression" priority="22" dxfId="7" stopIfTrue="1">
+      <formula>C60=""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M60:M74">
+    <cfRule type="expression" priority="23" dxfId="1">
+      <formula>M60&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L60:L74">
+    <cfRule type="expression" priority="24" dxfId="3">
+      <formula>L60&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -50010,7 +52280,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -50038,47 +52308,47 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="44" t="inlineStr">
+      <c r="A3" s="48" t="inlineStr">
         <is>
           <t>Property</t>
         </is>
       </c>
-      <c r="C3" s="44" t="inlineStr">
+      <c r="C3" s="48" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="E3" s="44" t="inlineStr">
+      <c r="E3" s="48" t="inlineStr">
         <is>
           <t>Renewal cycle</t>
         </is>
       </c>
-      <c r="G3" s="44" t="inlineStr">
+      <c r="G3" s="48" t="inlineStr">
         <is>
           <t>Auto-renew</t>
         </is>
       </c>
-      <c r="I3" s="44" t="inlineStr">
+      <c r="I3" s="48" t="inlineStr">
         <is>
           <t>Status (reference)</t>
         </is>
       </c>
-      <c r="K3" s="44" t="inlineStr">
+      <c r="K3" s="48" t="inlineStr">
         <is>
           <t>Property</t>
         </is>
       </c>
-      <c r="L3" s="44" t="inlineStr">
+      <c r="L3" s="48" t="inlineStr">
         <is>
           <t>Full name</t>
         </is>
       </c>
-      <c r="M3" s="44" t="inlineStr">
+      <c r="M3" s="48" t="inlineStr">
         <is>
           <t>Legal entity</t>
         </is>
       </c>
-      <c r="O3" s="44" t="inlineStr">
+      <c r="O3" s="48" t="inlineStr">
         <is>
           <t>Renew by</t>
         </is>

</xml_diff>